<commit_message>
Contacto = personal de apoyo (+1 809-252-7046), emergencias 911
</commit_message>
<xml_diff>
--- a/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
+++ b/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
@@ -1616,7 +1616,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>BORRADOR · verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>BORRADOR · verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>BORRADOR · verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1724,7 +1724,7 @@
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>BORRADOR · verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1762,7 +1762,7 @@
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>BORRADOR · verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2173,7 @@
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -2231,7 +2231,7 @@
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2289,7 +2289,7 @@
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2347,7 +2347,7 @@
       <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2453,7 +2453,7 @@
       <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       <c r="N15" s="3" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
       <c r="N16" s="3" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       <c r="N21" s="3" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       <c r="N24" s="3" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3334,7 @@
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
       <c r="N26" s="3" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3542,7 +3542,7 @@
       <c r="N29" s="3" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       <c r="N32" s="3" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3754,7 @@
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3852,7 +3852,7 @@
       <c r="N35" s="3" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
-          <t>BORRADOR · redactado con fuentes web (oct 2026), verificar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3905,7 @@
       <c r="N36" s="3" t="inlineStr"/>
       <c r="O36" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3958,7 @@
       <c r="N37" s="3" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4007,7 @@
       <c r="N38" s="3" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4060,7 @@
       <c r="N39" s="3" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       <c r="N40" s="3" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       <c r="N41" s="3" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       <c r="N42" s="3" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       <c r="N44" s="3" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       <c r="N45" s="3" t="inlineStr"/>
       <c r="O45" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       <c r="N46" s="3" t="inlineStr"/>
       <c r="O46" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4496,7 @@
       <c r="N47" s="3" t="inlineStr"/>
       <c r="O47" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4549,7 +4549,7 @@
       <c r="N48" s="3" t="inlineStr"/>
       <c r="O48" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       <c r="N49" s="3" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4659,7 @@
       <c r="N50" s="3" t="inlineStr"/>
       <c r="O50" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       <c r="N51" s="3" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4765,7 @@
       <c r="N52" s="3" t="inlineStr"/>
       <c r="O52" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       <c r="N53" s="3" t="inlineStr"/>
       <c r="O53" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       <c r="N54" s="3" t="inlineStr"/>
       <c r="O54" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       <c r="N55" s="3" t="inlineStr"/>
       <c r="O55" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       <c r="N56" s="3" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       <c r="N57" s="3" t="inlineStr"/>
       <c r="O57" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       <c r="N58" s="3" t="inlineStr"/>
       <c r="O58" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -5108,7 +5108,7 @@
       <c r="N59" s="3" t="inlineStr"/>
       <c r="O59" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -5161,7 +5161,7 @@
       <c r="N60" s="3" t="inlineStr"/>
       <c r="O60" t="inlineStr">
         <is>
-          <t>BORRADOR · genérico (solo datos del welcome pack), completar</t>
+          <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
     </row>
@@ -6077,12 +6077,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>1 (809) 697-6946</t>
+          <t>+1 809-252-7046</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Cómo se muestra</t>
+          <t>Teléfono del personal de apoyo (se muestra)</t>
         </is>
       </c>
     </row>
@@ -6094,12 +6094,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>+18096976946</t>
+          <t>+18092527046</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Número para el botón Llamar (con +1)</t>
+          <t>Número del botón Llamar (portada y Contacto)</t>
         </is>
       </c>
     </row>
@@ -6272,10 +6272,14 @@
           <t>emergencias_telefono</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>911</t>
+        </is>
+      </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>PENDIENTE: número que se muestra en Inicio. Si lo rellenas aparece el botón Llamar</t>
+          <t>Número del botón Llamar a emergencias</t>
         </is>
       </c>
     </row>
@@ -6290,7 +6294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6351,33 +6355,6 @@
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Confirmada por Miguel (oct 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>VMS2</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Villamisueno2</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>WPA</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Segunda red</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE: 07_QR/LEEME.md la asigna a Villa Bambú</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Emergencias: teléfonos y mapas con botones Llamar / Abrir en Google Maps
</commit_message>
<xml_diff>
--- a/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
+++ b/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
@@ -5282,7 +5282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5314,86 +5314,152 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Emergencias (9-1-1)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>911</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Centro Médico Jarabacoa</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr"/>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>+1 809-574-2431</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Jarabacoa%20Medical%20Center&amp;query_place_id=ChIJeQ-sXjcwsI4RM1DF4YnDoEM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Hospital Octavia Gautier de Vidal</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>+1 809-574-7179</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hospital%20Octavia%20Gautier%20de%20Vidal&amp;query_place_id=ChIJKziG6jYwsI4RheNkhTZ73PU</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Bomberos Buena Vista Jarabacoa</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>+1 809-574-6838</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Bomberos%20Buena%20Vista%20Jarabacoa&amp;query_place_id=ChIJbYIZDDYvsI4RnN55EkuW7t8</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Bomberos Jarabacoa</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>+1 809-574-4271</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Bomberos%20Jarabacoa&amp;query_place_id=ChIJn_KT7zYwsI4RlRHAmG-HkjI</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Policía Nacional</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>+1 809-574-7805 / +1 809-574-2540</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Cuartel%20Polic%C3%ADa%20Nacional%20Jarabacoa&amp;query_place_id=ChIJgV9B7jYwsI4R9dgM0ITzsyM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Digesett</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr"/>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>+1 809-574-7805</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=DIGESETT%20Comandancia%20Jarabacoa&amp;query_place_id=ChIJoWeZjTYwsI4RJg0VpsE3cnY</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Datos de Miguel (oct 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QR del Wi-Fi centrado verticalmente en la tarjeta
</commit_message>
<xml_diff>
--- a/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
+++ b/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
@@ -5324,7 +5324,6 @@
           <t>911</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Datos de Miguel (oct 2026)</t>
@@ -6413,11 +6412,7 @@
           <t>WPA</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Red principal</t>
-        </is>
-      </c>
+      <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Confirmada por Miguel (oct 2026)</t>

</xml_diff>

<commit_message>
Versión en inglés (/vms/en/): contenido desde columnas _en del Excel, interfaz traducida, selector ES/EN y detección del idioma del móvil
</commit_message>
<xml_diff>
--- a/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
+++ b/08_WELCOME_WEB/_datos/VMS_contenido.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,6 +552,16 @@
           <t>texto</t>
         </is>
       </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>titulo_en</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>texto_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -564,6 +574,16 @@
           <t>Para asegurar una estadía placentera, ofrecemos personal dedicado a la cocina, limpieza y asistencia para cualquier necesidad que pueda surgir durante tu estancia. Su horario es de 8:00 A.M. a 6:00 P.M.</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Support staff</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>To ensure a pleasant stay, we offer dedicated staff for cooking, cleaning, and assistance with any needs that may arise during your stay. Working hours: 8:00 A.M. – 6:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -576,6 +596,16 @@
           <t>Para cuidar el medio ambiente y ahorrar energía, te invitamos a disfrutar del aire puro de Jarabacoa y usar el aire acondicionado solo cuando sea necesario. Apaga las luces y el aire cuando no los uses. Juntos podemos disfrutar y cuidar el planeta.</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Temperature &amp; lights</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>To care for the environment and save energy, we invite you to enjoy the fresh air of Jarabacoa and use the air conditioning only when necessary. Please turn off the lights and air conditioning when not in use. Together, we can enjoy and care for the planet.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -588,6 +618,16 @@
           <t>Disponemos de un dispensador con un botellón de agua para tu comodidad.</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>We have a water dispenser with a water jug for your convenience.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -600,6 +640,16 @@
           <t>Se proporcionará una toalla por cada huésped registrado, y se deberá devolver la misma cantidad al finalizar la estancia.</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Towels</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>One towel will be provided for each registered guest, and the same number must be returned at the end of the stay.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -610,6 +660,16 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Si notas alguna anomalía o situación que requiera atención en la casa, infórmanos y haremos lo posible por solucionarla rápidamente.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Notice anything?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>If you notice any issues or situations that require attention in the house, please inform us, and we will do our best to resolve it quickly to improve your stay.</t>
         </is>
       </c>
     </row>
@@ -624,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -648,6 +708,11 @@
           <t>texto</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>texto_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -665,6 +730,11 @@
           <t>No se permiten fiestas, orquestas ni DJs.</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>No parties, live bands or DJs.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -682,6 +752,11 @@
           <t>Horario antirruidos: 11:00 P.M. – 7:00 A.M.</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Quiet hours: 11:00 P.M. – 7:00 A.M.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -699,6 +774,11 @@
           <t>Prohibido fumar dentro de la casa.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No smoking inside the house.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -716,6 +796,11 @@
           <t>No mover los muebles ni darles otro uso.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Don't move the furniture or use it for other purposes.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -733,6 +818,11 @@
           <t>Llaves perdidas: US$ 50.00 de reposición.</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lost keys: US$ 50.00 replacement fee.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -750,6 +840,11 @@
           <t>Ducha previa y traje de baño (no algodón) obligatorios.</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Shower first; swimwear required (no cotton).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -767,6 +862,11 @@
           <t>No hay salvavidas: uso bajo tu propio riesgo.</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>No lifeguard on duty: use at your own risk.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -784,6 +884,11 @@
           <t>Niños siempre supervisados; hay chalecos salvavidas.</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Children must always be supervised; life jackets available.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -801,6 +906,11 @@
           <t>No lanzarse de cabeza, correr, comer, fumar ni usar vidrio.</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>No diving, running, eating, smoking or glass.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -818,6 +928,11 @@
           <t>Calentamiento incluido 2 h al día; cada 2 h extra, US$ 50.00.</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Heating included 2 h a day; each extra 2 h, US$ 50.00.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -835,6 +950,11 @@
           <t>Sin aceites, lociones ni otros productos.</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>No oils, lotions or other products.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -852,6 +972,11 @@
           <t>Pide jacuzzi, fogata o BBQ al personal antes de las 5:00 P.M.</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Request the jacuzzi, fire pit or BBQ from the staff before 5:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -869,6 +994,11 @@
           <t>Somos pet friendly: mascotas pequeñas o medianas.</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>We're pet friendly: small or medium-sized pets.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -886,6 +1016,11 @@
           <t>No en muebles, camas, piscina ni jacuzzi.</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Not on furniture, beds, pool or jacuzzi.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -901,6 +1036,11 @@
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Recoge sus desechos y mantenlas vigiladas.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Pick up after them and keep them supervised.</t>
         </is>
       </c>
     </row>
@@ -915,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -939,6 +1079,16 @@
           <t>texto</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>grupo_en</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>texto_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -956,6 +1106,16 @@
           <t>No se permiten fiestas (no orquestas ni DJs).</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Parties are not allowed (no live bands or DJs).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -973,6 +1133,16 @@
           <t>Prohibido fumar dentro de la casa.</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Smoking is strictly prohibited inside the house.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -990,6 +1160,16 @@
           <t>No se permiten sustancias ilegales en las instalaciones.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Illegal substances are not permitted on the premises.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1007,6 +1187,16 @@
           <t>Todos los huéspedes deben estar registrados y proporcionar su identificación al menos 48 h antes del check-in.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>All guests must be registered and must provide valid identification at least 48 hours prior to check-in.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1024,6 +1214,16 @@
           <t>Máximo de 18 huéspedes.</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Maximum occupancy: 18 guests.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1041,6 +1241,16 @@
           <t>No se permiten fotografías ni vídeos comerciales sin previa autorización del propietario.</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Commercial photography or video recording is not allowed without prior authorization from the owner.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1058,6 +1268,16 @@
           <t>Respetar el horario «antirruidos» de la comunidad de Mata de Plátano, de 11:00 P.M. a 7:00 A.M., y en todo momento los niveles de decibeles permitidos por la legislación nacional (no exceder 60 dB de día y 50 dB de noche). No se permiten bocinas grandes.</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Please respect the community quiet hours in Mata de Plátano, from 11:00 P.M. to 7:00 A.M., and always comply with the noise levels established by national regulations (maximum 60 decibels during the day and 50 decibels at night). Large speakers are not permitted.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1075,6 +1295,16 @@
           <t>No mover los muebles ni darles un uso distinto al diseñado, tanto en interiores como en exteriores.</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Furniture must not be moved or used for purposes other than those intended, both indoors and outdoors.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1092,6 +1322,16 @@
           <t>Apaga el aire acondicionado y las luces cuando salgas.</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Please turn off air conditioning units and lights when leaving the property.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1109,6 +1349,16 @@
           <t>Respeta los horarios de entrada y salida.</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Respect check-in and check-out times.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1126,6 +1376,16 @@
           <t>Cuida tus llaves: las llaves perdidas tienen un costo de reemplazo de US$ 50.00.</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Take care of the keys; lost keys will incur a US$ 50.00 replacement fee.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1143,6 +1403,16 @@
           <t>Villa Mi Sueño es adecuada para niños menores de 12 años, que deben estar bajo supervisión de un adulto en todo momento.</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Specific rules</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Villa Mi Sueño is suitable for children under 12 years old; however, they must be under adult supervision at all times.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1160,6 +1430,16 @@
           <t>No coloques sobre la mesa de billar objetos que no le pertenezcan.</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Specific rules</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Do not place any objects on the pool table that do not belong to it.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1177,6 +1457,16 @@
           <t>No se permite instalar decoraciones que requieran perforaciones, cinta adhesiva u otros métodos que dañen las superficies.</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Specific rules</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Decorations that require drilling, adhesive tape, or any other methods that may damage surfaces are not permitted.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1194,6 +1484,16 @@
           <t>Profundidad de la piscina: 4 y 5 pies.</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pool depth: 4 and 5 feet.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1211,6 +1511,16 @@
           <t>Ducha obligatoria antes de entrar a la piscina o jacuzzi.</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Mandatory shower: a shower is required before entering the pool or jacuzzi.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1228,6 +1538,16 @@
           <t>Traje de baño obligatorio: no tejidos de algodón.</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Swimwear required: no cotton fabrics allowed.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1245,6 +1565,16 @@
           <t>No hay personal salvavidas en servicio. Los huéspedes usan las instalaciones bajo su propio riesgo.</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>There are no lifeguards on duty. Guests use the facilities at their own risk.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1262,6 +1592,16 @@
           <t>Los niños deben ser supervisados por un adulto en todo momento. Tenemos chalecos salvavidas disponibles para los más pequeños.</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Children must be supervised by an adult at all times. For your safety and peace of mind, we have life jackets available for the little ones.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1279,6 +1619,16 @@
           <t>No correr ni saltar en el área de la piscina.</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No running or jumping in the pool area.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1296,6 +1646,16 @@
           <t>No lanzarse de cabeza a la piscina o jacuzzi.</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No diving headfirst into the pool or jacuzzi.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1313,6 +1673,16 @@
           <t>No consumir alimentos en el área.</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No eating in the pool area.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1330,6 +1700,16 @@
           <t>No fumar.</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No smoking.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1347,6 +1727,16 @@
           <t>No usar vidrio ni objetos pequeños dentro de la piscina.</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>No glass or small objects in the pool.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1364,6 +1754,16 @@
           <t>No usar aceites, lociones u otros productos en el jacuzzi.</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>No oils, lotions, or other products in the jacuzzi.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1381,6 +1781,16 @@
           <t>Mantener el volumen bajo y evitar comportamientos ruidosos.</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Keep the volume low and avoid loud behavior.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1398,6 +1808,16 @@
           <t>No se permiten mascotas en la piscina o jacuzzi.</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>No pets allowed in the pool or jacuzzi.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1415,6 +1835,16 @@
           <t>Visitas solo con consentimiento previo del anfitrión.</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Visitors are allowed only with prior consent from the host.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1432,6 +1862,16 @@
           <t>El precio incluye la climatización del jacuzzi por 2 h diarias. Si quieres calentarlo más tiempo, cada 2 h adicionales cuestan US$ 50.00. Tanto el calentamiento incluido como el adicional deben notificarse al personal antes de las 5:00 P.M.</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Additional information</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>The price includes jacuzzi heating for 2 hours per day. If you wish to heat it for a longer period, an additional fee of US$ 50.00 applies for every extra 2 hours. Both the included heating time and any additional heating must be requested from the staff before 5:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1449,6 +1889,16 @@
           <t>Tenemos disponible fogata y BBQ. La leña está incluida en el precio; si prefieres usar carbón, debes traerlo. Solicita la fogata o el BBQ al personal antes de las 5:00 P.M.</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Additional information</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>A fire pit and BBQ are available. Firewood is included in the price; if you prefer charcoal, please bring it. If you would like to use the fire pit or the BBQ, please request it from the staff before 5:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1466,6 +1916,16 @@
           <t>Aceptamos con gusto hasta un máximo de 2 mascotas de tamaño pequeño y mediano.</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>We happily accept up to 2 small or medium-sized pets.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1483,6 +1943,16 @@
           <t>No se permiten mascotas en los muebles, camas, piscina o jacuzzi.</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pets are not allowed on furniture, beds, or in the pool or jacuzzi.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1500,6 +1970,16 @@
           <t>Asegúrate de manejar los desechos correctamente y mantener el área exterior limpia.</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Please dispose of pet waste properly and keep the outdoor area clean.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1515,6 +1995,16 @@
       <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Mantén vigilada a tu mascota para prevenir accidentes o daños a la propiedad.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Supervise your pet to prevent accidents or damage to the property.</t>
         </is>
       </c>
     </row>
@@ -1529,7 +2019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1582,6 +2072,16 @@
           <t>credito_fotos</t>
         </is>
       </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>categoria_en</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>descripcion_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1619,6 +2119,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Paragliding</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Fly over the Jarabacoa valley. Check schedules, prices and requirements with each operator.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1652,6 +2162,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Buggies &amp; four-wheelers</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Buggy and ATV tours along mountain trails and rivers. Check routes and prices with each operator.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1694,6 +2214,16 @@
           <t>Starus · CC BY-SA 3.0 · Wikimedia Commons</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Rafting &amp; tubing</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Raft or tube down the rivers of Jarabacoa with a guide. Check the season and requirements.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1732,6 +2262,16 @@
           <t>Treeman · Public domain · Wikimedia Commons</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Hiking</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Hiking trails through the mountains. Choose yours on Wikiloc by level and distance.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1763,6 +2303,16 @@
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mountain biking</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Mountain bike routes around Jarabacoa, with maps and elevation on Wikiloc.</t>
         </is>
       </c>
     </row>
@@ -1786,6 +2336,11 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Supermarket</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1807,6 +2362,11 @@
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Grocery store</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1828,6 +2388,11 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Butcher shop</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1849,6 +2414,11 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1870,6 +2440,11 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Gas station</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1891,6 +2466,11 @@
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1912,6 +2492,11 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Shops</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1933,6 +2518,11 @@
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Church</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1954,6 +2544,11 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1966,7 +2561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P60"/>
+  <dimension ref="A1:S60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2066,6 +2661,21 @@
           <t>credito_fotos</t>
         </is>
       </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>categoria_en</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>subtitulo_en</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>descripcion_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2123,6 +2733,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>River swimming area less than 3 km away, inside Mata de Plátano</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>River swimming area less than 3 km from the villa, inside the Mata de Plátano residential area. Perfect for cooling off and spending the day in nature.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -2181,6 +2806,16 @@
           <t>Jos1950 · CC BY-SA 4.0 · Wikimedia Commons</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>One of Jarabacoa's most iconic waterfalls, with a huge rock wall as a backdrop. The way down has steep stretches and steps that can be slippery: wear shoes with good grip.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2239,6 +2874,16 @@
           <t>Phyrexian · CC BY-SA 4.0 · Wikimedia Commons</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>A waterfall of about 25 m that drops into a natural green pool where you can swim. It's reached by a short, flat trail through a canyon, with bridges and wooden steps. About 10 minutes by car from town.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2295,6 +2940,16 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>Jos1950 · CC BY-SA 4.0 · Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Park where the Jimenoa and Yaque del Norte rivers meet, with pools among the rocks and large lawns for a picnic. There's a snack bar and horse rental. About 10 minutes from town.</t>
         </is>
       </c>
     </row>
@@ -2348,6 +3003,16 @@
       <c r="O6" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Paragliding</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Paragliding school offering tandem flights with a pilot. You meet on Avenida Pedregal and ride a 4x4 up to the take-off point; the flight lasts about 15–30 minutes depending on the wind.</t>
         </is>
       </c>
     </row>
@@ -2403,6 +3068,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Paragliding</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Paragliding flights in Jarabacoa. Check availability, price and meeting point by phone or Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2456,6 +3131,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Paragliding</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Paragliding flights in Jarabacoa. Check availability, price and meeting point by phone or Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2505,6 +3190,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Buggies &amp; four-wheelers</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Buggy and ATV tours along Jarabacoa's trails. Book by phone or Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2554,6 +3249,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Buggies &amp; four-wheelers</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>ATV and buggy rental to explore Jarabacoa. Book by phone or Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2605,6 +3310,16 @@
       <c r="O11" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Rafting &amp; tubing</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Adventure center and hotel just over 1 km from downtown Jarabacoa. It runs rafting trips on the Yaque del Norte, the longest river in the Caribbean, as well as canyoning, horseback rides and mountain bike routes.</t>
         </is>
       </c>
     </row>
@@ -2660,6 +3375,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Rafting &amp; tubing</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Rafting and tubing on the rivers of Jarabacoa. Check departures and requirements by phone or Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2707,6 +3432,16 @@
       <c r="O13" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Rafting &amp; tubing</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Rafting and tubing in Jarabacoa. Check departures and requirements on Instagram.</t>
         </is>
       </c>
     </row>
@@ -2758,6 +3493,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Hiking</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>The best trails in Jarabacoa</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Hiking trails through the mountains of Jarabacoa, with map, distance and elevation. Jarabacoa is also the starting point for Pico Duarte, the highest peak in the Caribbean.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2807,6 +3557,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Mountain biking</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>In Jarabacoa</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Mountain bike routes around Jarabacoa on Wikiloc, with map, distance and elevation so you can choose by level.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2852,6 +3617,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>La Confluencia has horses for rent for family rides. There are also guided horseback tours through the countryside to Salto Baiguate.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2901,6 +3676,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>A stroll through downtown Jarabacoa: its streets, shops and cafés.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2958,6 +3743,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Petting zoo · farm animals</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Farm with animals to visit with the family, in the Ruta de las Flores area.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -3017,6 +3817,21 @@
       <c r="O19" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Seasonal only: check availability</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Rancho Baiguate's butterfly garden. Open only in season: check availability before you go.</t>
         </is>
       </c>
     </row>
@@ -3072,6 +3887,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Ice cream shop in Jarabacoa, perfect for a break during your walk around town.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -3127,6 +3952,21 @@
       <c r="O21" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Orchids and succulents</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Orchid and succulent nursery in Mata de Plátano, on the way to the villa. According to Julián and Deysi, they sell the most beautiful orchids in the country.</t>
         </is>
       </c>
     </row>
@@ -3182,6 +4022,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Relaxed plans</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Guided tours of its fields</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Guided tours of aromatic herb and vegetable plantations, with a restaurant that cooks with what's grown on the farm.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -3235,6 +4090,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>On the outskirts of Jarabacoa, surrounded by fields of aromatic herbs. Market cuisine with organic ingredients, ideal for brunch or a sunset cocktail; the visit includes a tour of the garden. Open Thursday to Sunday (check before you go).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -3284,6 +4149,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Restaurant at the Jarabacoa Country Club with signature Caribbean cuisine. Reservations recommended.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -3337,6 +4212,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Restaurant at the Ribera Country Club. Check hours and reservations by phone.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3390,6 +4275,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -3441,6 +4336,16 @@
       <c r="O27" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Signature cuisine by chef Adin Langille, combining local produce with techniques learned in New York restaurants. Mountain views.</t>
         </is>
       </c>
     </row>
@@ -3492,6 +4397,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check hours and reservations by phone.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3545,6 +4460,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Kitchen and grill in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3598,6 +4523,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3651,6 +4586,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3704,6 +4649,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>At the top of the Jamaca de Dios residential area, on the Palo Blanco road. Its highlight is the panoramic view over all of Jarabacoa, especially at dusk when the valley lights come on. The drive up is steep.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -3757,6 +4712,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Restaurant at Vista del Campo Country Club &amp; Villas, on the road to Salto de Jimenoa, past the golf course.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3810,6 +4775,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Restaurant at the Pinar Dorado hotel, in downtown Jarabacoa.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -3855,6 +4830,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Roadside restaurant famous in the valley for its wood-fired pork ribs, served with fried plantains.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -3908,6 +4893,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -3959,6 +4954,16 @@
       <c r="O37" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Café in Jarabacoa, a good option for coffee or breakfast. Check hours on Instagram.</t>
         </is>
       </c>
     </row>
@@ -4010,6 +5015,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Café in Jarabacoa. Check hours by phone.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4063,6 +5078,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -4116,6 +5141,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Restaurant in Jarabacoa. Check the menu and hours on Instagram.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -4169,6 +5204,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Pizzeria in Jarabacoa. Ask by phone if they deliver to Mata de Plátano.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -4220,6 +5265,16 @@
       <c r="O42" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Pizzeria in Jarabacoa. Ask by phone if they deliver to Mata de Plátano.</t>
         </is>
       </c>
     </row>
@@ -4279,6 +5334,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Grocery store</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Delivers to Villa Mi Sueño</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Grocery store (colmado) that delivers to Villa Mi Sueño: the easiest option for drinks, ice and the basics.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -4336,6 +5406,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Supermarket</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Av. Independencia</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Supermarket on Av. Independencia, Jarabacoa.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -4393,6 +5478,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Supermarket</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Main road</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Supermarket on the main road in Jarabacoa.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -4448,6 +5548,21 @@
       <c r="O46" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Supermarket</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Calle Obdulio Jiménez</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Supermarket on Calle Obdulio Jiménez, Jarabacoa.</t>
         </is>
       </c>
     </row>
@@ -4499,6 +5614,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Calle Marina Nelson Galán</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Jarabacoa's public market, on Calle Marina Nelson Galán: fruit, vegetables and local products.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -4552,6 +5682,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Butcher shop</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Butcher &amp; fish shop · delivery available</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Butcher and fish shop with delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -4605,6 +5750,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Butcher shop</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Butcher shop</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Butcher shop in Jarabacoa.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -4660,6 +5820,21 @@
       <c r="O50" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Shops</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Hardware store</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Hardware store and multi-store in Jarabacoa.</t>
         </is>
       </c>
     </row>
@@ -4715,6 +5890,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Shops</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>General goods</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>General goods store in Jarabacoa.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -4768,6 +5958,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Shops</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Clothing store in Jarabacoa.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -4821,6 +6026,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Av. Estela Geraldino No. 17</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Pharmacy on Av. Estela Geraldino No. 17.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -4870,6 +6090,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Pharmacy · Av. Independencia</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Pharmacy on Av. Independencia.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -4915,6 +6150,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Banco BHD branch in Jarabacoa. Check the exact location on the map.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -4960,6 +6205,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Banreservas branch in Jarabacoa. Check the exact location on the map.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -5005,6 +6260,16 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Banco Popular branch in Jarabacoa. Check the exact location on the map.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -5058,6 +6323,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Gas station</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Gas station · open 24 hours</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Gas station open 24 hours.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -5111,6 +6391,21 @@
           <t>Revisado por Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Gas station</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Gas station · open 24 hours</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Gas station open 24 hours.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -5162,6 +6457,21 @@
       <c r="O60" t="inlineStr">
         <is>
           <t>Revisado por Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Church</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>C. del Carmen, Jarabacoa</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Church on Calle Del Carmen, Jarabacoa.</t>
         </is>
       </c>
     </row>
@@ -5181,7 +6491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -5193,6 +6503,11 @@
           <t>paso</t>
         </is>
       </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>paso_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -5200,6 +6515,11 @@
           <t>Comenzamos desde el Cruce de Jarabacoa.</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>We start at the Jarabacoa crossroads.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -5207,6 +6527,11 @@
           <t>Pasarán la Bomba Texaco, Zona Franca, Bayacanes, Arepas de Maíz, La Virgencita, una subida GRANDE, Los Alpes Dominicanos, Parador de Jesús y Buena Vista (¡cuidado!, muchos lo confunden con Jarabacoa) hasta la Estación Shell. Aquí comienza la ruta hasta Villa Mi Sueño.</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>You'll pass the Texaco gas station, Zona Franca, Bayacanes, Arepas de Maíz, La Virgencita, a BIG hill, Los Alpes Dominicanos, Parador de Jesús and Buena Vista (careful! many people confuse it with Jarabacoa) until you reach the Shell station. This is where the route to Villa Mi Sueño begins.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -5214,6 +6539,11 @@
           <t>Al salir de la Estación Shell (siempre camino a Jarabacoa), busquen con cuidado el Cruce del Salto de Jimenoa (muchísimos letreros lo indican) y tomen a la izquierda.</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>After leaving the Shell station (always heading towards Jarabacoa), carefully look for the Salto de Jimenoa crossroads (there are plenty of signs) and turn left.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -5221,6 +6551,11 @@
           <t>Sigan la carretera hacia el Salto y, en la primera intersección en forma de Y, tomen a la izquierda.</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Follow the road towards the Salto and, at the first Y-shaped intersection, turn left.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -5228,6 +6563,11 @@
           <t>Pasan el Campo de Golf. Llegarán a una T: doblen a la derecha, siempre en dirección al Salto de Jimenoa.</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>You'll pass the golf course. You'll come to a T-junction: turn right, always in the direction of Salto de Jimenoa.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -5235,6 +6575,11 @@
           <t>Pasan el Hotel Montaña Azul. Atención: se acerca un cruce que dice Mata de Plátano; ahí tomen la izquierda. (Si siguen derecho llegarán al Salto y tendrán que devolverse.)</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>You'll pass the Montaña Azul Hotel. Careful: a crossroads with a sign for Mata de Plátano is coming up; turn left there. (If you keep going straight, you'll reach the Salto and will have to turn back.)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -5242,6 +6587,11 @@
           <t>Sigan este camino hasta la garita. Pueden preguntar a los guardianes cómo llegar a Villa Mi Sueño o a la casa de Julián y Deysi (¡seguro que les indican!), o seguir solos.</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Follow this road until you reach the security checkpoint (garita). You can ask the guards how to get to Villa Mi Sueño or to Julián and Deysi's house (they'll definitely give you directions!), or continue on your own.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -5249,6 +6599,11 @@
           <t>Tomen el Camino del Ébano, la calle principal de Mata de Plátano. Pasan un tanque azul de agua (sigan el camino que gira a la izquierda) y varias casas bonitas hasta Rancho Bariloche.</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Take Camino del Ébano, the main road through Mata de Plátano. You'll pass a blue water tank (follow the road that curves left) and several beautiful houses until you reach Rancho Bariloche.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -5256,6 +6611,11 @@
           <t>En Rancho Bariloche (¡ojo, hay un badén bien grande!) doblen a la derecha por el Camino del Nuez.</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>At Rancho Bariloche (watch out, there's a big dip in the road!) turn right onto Camino del Nuez.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -5263,11 +6623,21 @@
           <t>Sigan derecho por el Camino del Nuez: en la primera intersección giren a la derecha y en la segunda a la izquierda, tomando el Camino del Bambú.</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Continue straight on Camino del Nuez: at the first intersection turn right and at the second turn left, onto Camino del Bambú.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Sigan… sigan… ¡no se desesperen! Al final del Camino del Bambú, la última casa, está Villa Mi Sueño.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Keep going… keep going… don't lose patience! At the very end of Camino del Bambú, the last house, you'll find Villa Mi Sueño.</t>
         </is>
       </c>
     </row>
@@ -5282,7 +6652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5312,6 +6682,11 @@
           <t>nota</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>nombre_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5329,6 +6704,11 @@
           <t>Datos de Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Emergency (9-1-1)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5351,6 +6731,11 @@
           <t>Datos de Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Jarabacoa Medical Center</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5395,6 +6780,11 @@
           <t>Datos de Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Buena Vista Fire Department (Jarabacoa)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5417,6 +6807,11 @@
           <t>Datos de Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Jarabacoa Fire Department</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5439,6 +6834,11 @@
           <t>Datos de Miguel (oct 2026)</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>National Police</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5459,6 +6859,11 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>Datos de Miguel (oct 2026)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Digesett (traffic police)</t>
         </is>
       </c>
     </row>
@@ -5973,7 +7378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5997,6 +7402,11 @@
           <t>explicación</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>valor_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6048,6 +7458,11 @@
           <t>Línea de ubicación en portada</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Jarabacoa · Dominican Republic</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -6201,6 +7616,11 @@
           <t>Mensaje que aparece escrito al abrir el chat</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Hi, I'm a guest at Villa Mi Sueño.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -6240,6 +7660,11 @@
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Julián and Deysi</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -6430,7 +7855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6448,6 +7873,11 @@
           <t>texto</t>
         </is>
       </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>texto_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6460,6 +7890,11 @@
           <t>Bienvenidos</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -6472,6 +7907,11 @@
           <t>Bienvenidos a nuestra casa</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Welcome to our home</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -6484,6 +7924,11 @@
           <t>Todo lo que necesitas para disfrutar tu estadía, en un solo lugar.</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Everything you need to enjoy your stay, all in one place.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -6496,6 +7941,11 @@
           <t>Tu guía</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Your guide</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -6508,6 +7958,11 @@
           <t>¡Bienvenido a Villa Mi Sueño! Estamos muy felices de que hayas elegido hospedarte con nosotros. Queremos que te sientas cómodo y como en casa, sin importar la distancia.</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Welcome to Villa Mi Sueño! We are so happy that you chose to stay with us. We want you to feel comfortable and at home, no matter the distance.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -6520,6 +7975,11 @@
           <t>Todo el equipo de Villa Mi Sueño y Hospedify te desea una experiencia maravillosa. ¡Disfruta cada momento aquí!</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The entire team at Villa Mi Sueño and Hospedify wishes you a wonderful experience. Enjoy every moment here!</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -6532,6 +7992,11 @@
           <t>Si le preguntas a Julián y a Deysi qué es Villa Mi Sueño, te dirán que es su rincón especial, un lugar lleno de magia y amor donde han creado recuerdos inolvidables con su familia, especialmente con sus nietos.</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>If you ask Julián and Deysi what Villa Mi Sueño is, they will tell you that it's their special corner, a place full of magic and love where they have created unforgettable memories with their family, especially with their grandchildren.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -6544,6 +8009,11 @@
           <t>Cada rincón de este refugio ha sido pensado con detalle y cuidado, para que te sientas como en casa desde el primer momento. Nos encanta disfrutar de la buena comida, la música, un buen vino, y esos momentos tranquilos con un libro en la mano, acompañados de un cafecito o un chocolate caliente.</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Every corner of this retreat has been thoughtfully and carefully designed so you feel at home from the very first moment. We love enjoying good food, music, a fine wine, and those peaceful moments with a book in hand, accompanied by a little coffee or hot chocolate.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -6556,6 +8026,11 @@
           <t>Hoy queremos abrirte las puertas de nuestro pequeño paraíso para que tú también puedas vivir momentos únicos, rodeado de la misma calidez y cariño con los que fue creado. ¡Esperamos que te sientas parte de nuestra familia y que disfrutes cada instante aquí!</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Today, we want to open the doors to our little paradise so you can also experience unique moments, surrounded by the same warmth and love with which it was created. We hope you feel part of our family and enjoy every moment here!</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -6568,6 +8043,11 @@
           <t>Etiqueta #VillaMiSueño y comparte tus momentos favoritos con nosotros. ¡Siempre nos emociona y nos encanta ver las experiencias de nuestros huéspedes!</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Tag #VillaMiSueño and share your favorite moments with us. We're always thrilled to see our guests' experiences!</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -6580,6 +8060,11 @@
           <t>Agradecemos mucho a nuestros huéspedes por tomarse el tiempo de evaluarnos. Te mandamos una breve encuesta a tu salida.</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>We greatly appreciate our guests for taking the time to leave a review. We'll send you a short survey after your stay.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -6592,6 +8077,11 @@
           <t>The Return Stay Club</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The Return Stay Club</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -6604,6 +8094,11 @@
           <t>Obtén una noche gratis en tu quinta estancia. Valoramos a nuestros huéspedes que nos eligen una y otra vez: cada vez que regreses disfrutarás de aún más beneficios y descuentos.</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Enjoy a free night on your fifth stay! We deeply value our guests who choose to stay with us time and again: each time you return, you'll enjoy even more perks and discounts.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -6616,6 +8111,11 @@
           <t>Escanea el código para acceder</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Scan the code to connect</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6628,6 +8128,11 @@
           <t>En caso de emergencias</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>In case of emergency</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -6640,6 +8145,11 @@
           <t>El botiquín está en el cajón inferior del mueble sideboard de la sala.</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>The first aid kit is in the bottom drawer of the sideboard in the living room.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -6652,6 +8162,11 @@
           <t>Los extintores están en las áreas de circulación.</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Fire extinguishers are located in the circulation areas.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -6664,6 +8179,11 @@
           <t>Centro Médico Jarabacoa · Hospital Octavia Gautier de Vidal · Bomberos · Policía · Digesett</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Jarabacoa Medical Center · Hospital Octavia Gautier de Vidal · Fire department · Police · Digesett</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -6676,6 +8196,11 @@
           <t>Estadía</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Your stay</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -6688,6 +8213,11 @@
           <t>Siéntete en casa</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Make yourself at home</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -6700,6 +8230,11 @@
           <t>Horarios, accesos y todo lo que la villa tiene para ti.</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Schedules, access and everything the villa has for you.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -6712,6 +8247,11 @@
           <t>Sabemos que los planes de viaje pueden cambiar. Si necesitas ajustar tu hora de llegada, contáctanos y haremos lo posible por adaptarnos a tu horario.</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>We know travel plans can change. If you need to adjust your arrival time, please contact us, and we will do our best to accommodate your schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -6724,6 +8264,11 @@
           <t>Hacemos nuestro mejor esfuerzo para acomodar salidas tardías, así que contáctanos si lo necesitas.</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>We make every effort to accommodate late check-outs, so please reach out if you need it.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -6736,6 +8281,11 @@
           <t>No olvides traer</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Don't forget to bring</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -6748,6 +8298,11 @@
           <t>Tráelo contigo o cómpralo de camino a la villa.</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Bring it with you or buy it on your way to the villa.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -6760,6 +8315,11 @@
           <t>Cocina, limpieza y asistencia para cualquier necesidad durante tu estancia.</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Cooking, cleaning and assistance with anything you need during your stay.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -6772,6 +8332,11 @@
           <t>Tu espacio, tu ritmo</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Your space, your pace</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -6784,6 +8349,11 @@
           <t>Días de piscina, noches junto al fuego.</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pool days, nights by the fire.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -6796,6 +8366,11 @@
           <t>Tenemos para ti</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>We have for you</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -6808,6 +8383,11 @@
           <t>También tenemos gazebo, patio privado, estacionamiento, espacio de oficina y comedor exterior para 8.</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>We also have a gazebo, a private patio, parking, an office space and an outdoor dining table for 8.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -6820,6 +8400,11 @@
           <t>Convivencia</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Living together</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -6832,6 +8417,11 @@
           <t>Cuidemos este lugar</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Let's take care of this place</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -6844,6 +8434,11 @@
           <t>¡Estás a punto de disfrutar de un hogar único! Cuídalo con el mismo cariño que tu propio espacio.</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>You're about to enjoy a unique home! Take care of it with the same love as your own space.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -6856,6 +8451,11 @@
           <t>Huéspedes registrados</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Registered guests</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -6868,6 +8468,11 @@
           <t>Identificación de todos al menos 48 h antes del check-in.</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ID for every guest at least 48 hours before check-in.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -6880,6 +8485,11 @@
           <t>Zonas de agua</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Water areas</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -6892,6 +8502,11 @@
           <t>Disfruta con calma y seguridad.</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Enjoy calmly and safely.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -6904,6 +8519,11 @@
           <t>4 y 5 pies</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>4 and 5 feet</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -6916,6 +8536,11 @@
           <t>2 h incluidas</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2 h included</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -6928,6 +8553,11 @@
           <t>Máximo 2</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Max. 2</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -6940,6 +8570,11 @@
           <t>¡Damos la bienvenida a tus mascotas y esperamos que se sientan también como en casa! Para garantizar una estancia estupenda para todos, aquí tienes algunos recordatorios para mantener nuestro espacio impecable.</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>We welcome your pets and hope they feel at home here, too! To ensure a wonderful stay for everyone, here are some pet etiquette reminders to help keep our space pristine for future guests.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -6952,6 +8587,11 @@
           <t>Jarabacoa</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Jarabacoa</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -6964,6 +8604,11 @@
           <t>Qué hacer</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -6976,6 +8621,11 @@
           <t>Ríos, montañas y sabores locales: una selección para explorar a tu propio ritmo.</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Rivers, mountains and local flavors: a selection to explore at your own pace.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -6988,6 +8638,11 @@
           <t>Naturaleza viva</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Living nature</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -7000,6 +8655,11 @@
           <t>Saltos, ríos y montaña</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Waterfalls, rivers and mountains</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -7012,6 +8672,11 @@
           <t>El balneario del río Camú está a menos de 3 km, dentro de Mata de Plátano. En la foto, el Salto Jimenoa.</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>The Camú River swimming area is less than 3 km away, inside Mata de Plátano. In the photo, Salto Jimenoa.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -7024,6 +8689,11 @@
           <t>Dónde comer</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Where to eat</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -7034,6 +8704,11 @@
       <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Directorio local</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Local directory</t>
         </is>
       </c>
     </row>
@@ -7060,7 +8735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7084,6 +8759,11 @@
           <t>destino</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>etiqueta_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7101,6 +8781,11 @@
           <t>casa</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Check-in</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -7118,6 +8803,11 @@
           <t>inicio/anfitriones</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>About the house</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -7135,6 +8825,11 @@
           <t>inicio/llegar</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Directions</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -7152,6 +8847,11 @@
           <t>inicio:wifi</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Wi-Fi</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -7169,6 +8869,11 @@
           <t>reglas</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>House rules</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -7186,6 +8891,11 @@
           <t>casa/debes</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Things to know</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -7203,6 +8913,11 @@
           <t>casa:tenemos</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Amenities</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -7220,6 +8935,11 @@
           <t>inicio/emergencias</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -7237,6 +8957,11 @@
           <t>explora</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Things to do</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -7254,6 +8979,11 @@
           <t>explora:comer</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Food &amp; drink</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -7271,6 +9001,11 @@
           <t>explora/directorio</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -7288,6 +9023,11 @@
           <t>explora:directorio</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Local directory</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -7305,6 +9045,11 @@
           <t>casa:checkout</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Before you leave</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -7322,6 +9067,11 @@
           <t>inicio/anfitriones</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Share &amp; Review</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -7337,6 +9087,11 @@
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>inicio/anfitriones</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Thank you</t>
         </is>
       </c>
     </row>
@@ -7351,7 +9106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7375,6 +9130,11 @@
           <t>en_tarjeta</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>texto_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7392,6 +9152,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>If you arrive at the scheduled time, the Villa Mi Sueño staff will welcome you.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -7409,6 +9174,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>If you arrive later, we will send the access code to your phone a few hours before.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -7426,6 +9196,11 @@
           <t>no</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>If you arrive in the dark, a flashlight will be helpful.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -7443,6 +9218,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Turn off all lights and appliances.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -7460,6 +9240,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Take the trash out to the containers.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -7475,6 +9260,11 @@
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>sí</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Hang the house key next to the front door.</t>
         </is>
       </c>
     </row>
@@ -7494,7 +9284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -7512,6 +9302,11 @@
           <t>tipo</t>
         </is>
       </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>item_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7524,6 +9319,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Toothpaste</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -7536,6 +9336,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Shampoo</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -7548,6 +9353,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Conditioner</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -7560,6 +9370,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Waterproof or hiking boots</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -7572,6 +9387,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -7584,6 +9404,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Books</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -7596,6 +9421,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bug repellent</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -7608,6 +9438,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Your food</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -7620,6 +9455,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Your drinks</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -7632,6 +9472,11 @@
           <t>básico</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -7644,6 +9489,11 @@
           <t>actitud</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Relaxation and enjoyment mindset :)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -7656,6 +9506,11 @@
           <t>actitud</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Adventurous spirit</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -7666,6 +9521,11 @@
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>actitud</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Connection with the senses</t>
         </is>
       </c>
     </row>
@@ -7680,7 +9540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7716,6 +9576,16 @@
           <t>en_resumen</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>etiqueta_en</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>descripcion_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7743,6 +9613,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>6 queen + 6 twin beds</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>6 queen-size double beds and 6 twin-size single beds, with pillows, blankets and bed linens.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -7770,6 +9650,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A/C in 5 bedrooms</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Air conditioning in 5 bedrooms. Please use it only when needed and turn it off when you leave.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -7797,6 +9687,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>7 bathrooms with hot water</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>7 equipped bathrooms with hot water, towels, bath mats and shower gel.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -7824,6 +9724,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Saltwater pool</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Saltwater pool, free of harmful chemicals. Depths of 4 and 5 feet.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -7851,6 +9761,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Heated jacuzzi</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Heating included 2 hours a day. Request it from the staff before 5:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -7878,6 +9798,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Fire pit with firewood</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Fire pit area with firewood included. Request it from the staff before 5:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -7905,6 +9835,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BBQ</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>BBQ with its tools. If you prefer charcoal, please bring your own. Request it before 5:00 P.M.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -7932,6 +9872,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Equipped kitchen</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Stove, gas oven, refrigerator, microwave, water dispenser, air fryer, blender, toaster, dishware and utensils.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -7959,6 +9909,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Wood-fired oven &amp; Lorena stove</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Wood-fired oven and Lorena stove.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -7986,6 +9946,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Dining for 12</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Dining table for 12 people.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -8013,6 +9983,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Pool table</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Pool table. Please don't place objects on it that don't belong to it.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -8040,6 +10020,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Treehouse</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Treehouse.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -8067,6 +10057,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Play area</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Play area.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -8090,6 +10090,16 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Baby items</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Baby chair, bassinet, playpen, baby bathtub and changing table.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -8117,6 +10127,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Gazebo</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Gazebo.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -8144,6 +10164,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Private patio</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Private patio.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -8171,6 +10201,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Outdoor dining</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Outdoor dining table for 8 people.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -8194,6 +10234,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Office space</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Desk and office chair.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -8221,6 +10271,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Parking space.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8248,6 +10308,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Living room</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Living room.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8275,6 +10345,16 @@
           <t>no</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Gardens and views</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Gardens and views of the Jarabacoa mountains.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8300,6 +10380,16 @@
       <c r="E23" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Mural</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>The villa's colorful mural.</t>
         </is>
       </c>
     </row>
@@ -8319,7 +10409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8337,6 +10427,16 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>grupo_en</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>item_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -8349,6 +10449,16 @@
           <t>Estufa</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Stove</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -8361,6 +10471,16 @@
           <t>Horno a gas</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Gas oven</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -8373,6 +10493,16 @@
           <t>Refrigerador, microondas y bebedero</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Refrigerator, microwave and water dispenser</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -8385,6 +10515,16 @@
           <t>Airfryer, licuadora y tostadora</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Air fryer, blender and toaster</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -8397,6 +10537,16 @@
           <t>Horno a leña y Lorena</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Wood-fired oven and Lorena stove</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -8409,6 +10559,16 @@
           <t>Vajilla, tazas, platos y cubiertos</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dishware, cups, plates and cutlery</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -8421,6 +10581,16 @@
           <t>Accesorios y utensilios de cocina</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Kitchen accessories and utensils</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -8433,6 +10603,16 @@
           <t>Mesa de comedor para 12 personas</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Dining table for 12 people</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -8445,6 +10625,16 @@
           <t>6 camas dobles tamaño queen</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bedrooms</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>6 queen-size double beds</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -8457,6 +10647,16 @@
           <t>6 camas individuales tamaño twin</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Bedrooms</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>6 twin-size single beds</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -8469,6 +10669,16 @@
           <t>Aire acondicionado en 5 habitaciones</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Bedrooms</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Air conditioning in 5 bedrooms</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -8481,6 +10691,16 @@
           <t>Almohadas, mantas y ropa de cama</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bedrooms</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Pillows, blankets and bed linens</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -8493,6 +10713,16 @@
           <t>7 baños equipados</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Bathrooms</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>7 equipped bathrooms</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -8505,6 +10735,16 @@
           <t>Agua caliente</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Bathrooms</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hot water</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -8517,6 +10757,16 @@
           <t>Toallas y alfombras de baño</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Bathrooms</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Towels and bath mats</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -8529,6 +10779,16 @@
           <t>Gel de baño</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Bathrooms</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Shower gel</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -8541,6 +10801,16 @@
           <t>BBQ y sus herramientas</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BBQ and its tools</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -8553,6 +10823,16 @@
           <t>Mesa de comedor para 8 personas</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Dining table for 8 people</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -8565,6 +10845,16 @@
           <t>Patio privado</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Private patio</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -8577,6 +10867,16 @@
           <t>Área para fogata con leña</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fire pit area with firewood</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -8589,6 +10889,16 @@
           <t>Piscina de cloración salina: libre de químicos nocivos</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Saltwater pool: free of harmful chemicals</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -8601,6 +10911,16 @@
           <t>Jacuzzi con calentador</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Jacuzzi with heater</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -8613,6 +10933,16 @@
           <t>Casa del árbol</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Treehouse</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -8625,6 +10955,16 @@
           <t>Área de juegos</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Play area</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -8637,6 +10977,16 @@
           <t>Espacio para estacionar</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Parking space</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -8649,6 +10999,16 @@
           <t>Gazebo</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Gazebo</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -8661,6 +11021,16 @@
           <t>Mesa de billar</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Outdoors</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Pool table</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -8673,6 +11043,16 @@
           <t>Escritorio y silla de trabajo</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Office space</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Desk and office chair</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -8685,6 +11065,16 @@
           <t>Silla para bebé</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>For babies</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Baby chair</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -8697,6 +11087,16 @@
           <t>Moisés para bebé</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>For babies</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Baby bassinet</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -8709,6 +11109,16 @@
           <t>Corral</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>For babies</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Playpen</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -8721,6 +11131,16 @@
           <t>Bañito</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>For babies</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Baby bathtub</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -8731,6 +11151,16 @@
       <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Cambiador</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>For babies</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Changing table</t>
         </is>
       </c>
     </row>

</xml_diff>